<commit_message>
delete unnecessary files and test successfully
</commit_message>
<xml_diff>
--- a/need/引脚对照表.xlsx
+++ b/need/引脚对照表.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FpgaProject\XilinxProject\XC7A35T\fir_interpolation\need\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{564FC7D9-B0DA-46B5-9B41-C1586FA4AB8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D622909-B370-419B-91E8-A1659977ADF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="-528" windowWidth="30984" windowHeight="18600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="102">
   <si>
     <t>自制板子</t>
   </si>
@@ -330,6 +330,22 @@
   </si>
   <si>
     <t>P17</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Y18</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>蜂鸣器</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>AB18</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Buzzer</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
@@ -337,7 +353,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -399,8 +415,30 @@
       <family val="2"/>
       <charset val="134"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="黑体"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Adobe 黑体 Std R"/>
+      <family val="2"/>
+      <charset val="128"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -440,6 +478,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -530,7 +574,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -610,6 +654,18 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -880,19 +936,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:G88"/>
+  <dimension ref="A1:H88"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.33203125" customWidth="1"/>
-    <col min="2" max="2" width="7.33203125" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="15.33203125" customWidth="1"/>
+    <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.33203125" customWidth="1"/>
+    <col min="3" max="3" width="34.5546875" customWidth="1"/>
     <col min="4" max="4" width="18.33203125" customWidth="1"/>
     <col min="5" max="5" width="17.44140625" customWidth="1"/>
     <col min="6" max="6" width="9" style="1"/>
     <col min="7" max="7" width="9" style="2"/>
+    <col min="8" max="8" width="9" style="28"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="40.799999999999997" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="40.799999999999997" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -903,7 +960,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="12" t="s">
@@ -921,8 +978,11 @@
       <c r="G2" s="16" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H2" s="29" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="17"/>
       <c r="B3" s="17"/>
       <c r="C3" s="18" t="s">
@@ -937,7 +997,7 @@
       <c r="F3" s="20"/>
       <c r="G3" s="21"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="22" t="s">
         <v>11</v>
       </c>
@@ -952,7 +1012,7 @@
       <c r="F4" s="20"/>
       <c r="G4" s="21"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="22" t="s">
         <v>14</v>
       </c>
@@ -967,7 +1027,7 @@
       <c r="F5" s="20"/>
       <c r="G5" s="21"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="22" t="s">
         <v>16</v>
       </c>
@@ -982,7 +1042,7 @@
       <c r="F6" s="20"/>
       <c r="G6" s="21"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="22" t="s">
         <v>18</v>
       </c>
@@ -997,7 +1057,7 @@
       <c r="F7" s="20"/>
       <c r="G7" s="21"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="22" t="s">
         <v>20</v>
       </c>
@@ -1012,7 +1072,7 @@
       <c r="F8" s="20"/>
       <c r="G8" s="21"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="22" t="s">
         <v>22</v>
       </c>
@@ -1027,7 +1087,7 @@
       <c r="F9" s="20"/>
       <c r="G9" s="21"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="22" t="s">
         <v>24</v>
       </c>
@@ -1042,7 +1102,7 @@
       <c r="F10" s="20"/>
       <c r="G10" s="21"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="22" t="s">
         <v>26</v>
       </c>
@@ -1057,7 +1117,7 @@
       <c r="F11" s="20"/>
       <c r="G11" s="21"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="22" t="s">
         <v>28</v>
       </c>
@@ -1072,7 +1132,7 @@
       <c r="F12" s="20"/>
       <c r="G12" s="21"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="22" t="s">
         <v>30</v>
       </c>
@@ -1087,7 +1147,7 @@
       <c r="F13" s="20"/>
       <c r="G13" s="21"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="22" t="s">
         <v>33</v>
       </c>
@@ -1102,7 +1162,7 @@
       <c r="F14" s="20"/>
       <c r="G14" s="21"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="22" t="s">
         <v>35</v>
       </c>
@@ -1117,7 +1177,7 @@
       <c r="F15" s="20"/>
       <c r="G15" s="21"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="22" t="s">
         <v>37</v>
       </c>
@@ -1166,7 +1226,9 @@
       <c r="A19" s="22" t="s">
         <v>44</v>
       </c>
-      <c r="B19" s="22"/>
+      <c r="B19" s="27" t="s">
+        <v>98</v>
+      </c>
       <c r="C19" s="23"/>
       <c r="D19" s="24"/>
       <c r="E19" s="25"/>
@@ -1358,7 +1420,7 @@
       <c r="F32" s="20"/>
       <c r="G32" s="21"/>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="22" t="s">
         <v>67</v>
       </c>
@@ -1373,7 +1435,7 @@
       <c r="F33" s="20"/>
       <c r="G33" s="21"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="22" t="s">
         <v>69</v>
       </c>
@@ -1388,7 +1450,7 @@
       <c r="F34" s="20"/>
       <c r="G34" s="21"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="22" t="s">
         <v>71</v>
       </c>
@@ -1403,7 +1465,7 @@
       <c r="F35" s="20"/>
       <c r="G35" s="21"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="22" t="s">
         <v>73</v>
       </c>
@@ -1418,7 +1480,7 @@
       <c r="F36" s="20"/>
       <c r="G36" s="21"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="22" t="s">
         <v>75</v>
       </c>
@@ -1433,7 +1495,7 @@
       <c r="F37" s="20"/>
       <c r="G37" s="21"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="22" t="s">
         <v>77</v>
       </c>
@@ -1448,7 +1510,7 @@
       <c r="F38" s="20"/>
       <c r="G38" s="21"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="22" t="s">
         <v>79</v>
       </c>
@@ -1463,7 +1525,7 @@
       <c r="F39" s="20"/>
       <c r="G39" s="21"/>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="22" t="s">
         <v>81</v>
       </c>
@@ -1478,7 +1540,7 @@
       <c r="F40" s="20"/>
       <c r="G40" s="21"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="22" t="s">
         <v>83</v>
       </c>
@@ -1493,7 +1555,7 @@
       <c r="F41" s="20"/>
       <c r="G41" s="21"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="22" t="s">
         <v>85</v>
       </c>
@@ -1508,7 +1570,7 @@
       <c r="F42" s="20"/>
       <c r="G42" s="21"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="22" t="s">
         <v>87</v>
       </c>
@@ -1523,7 +1585,7 @@
       <c r="F43" s="20"/>
       <c r="G43" s="21"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="22" t="s">
         <v>89</v>
       </c>
@@ -1538,28 +1600,33 @@
       <c r="F44" s="20"/>
       <c r="G44" s="21"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="8"/>
-      <c r="B45" s="8"/>
+      <c r="B45" s="22" t="s">
+        <v>100</v>
+      </c>
       <c r="C45" s="7"/>
       <c r="D45" s="5"/>
       <c r="E45" s="6"/>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H45" s="30" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" s="8"/>
       <c r="B46" s="8"/>
       <c r="C46" s="7"/>
       <c r="D46" s="5"/>
       <c r="E46" s="6"/>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" s="8"/>
       <c r="B47" s="8"/>
       <c r="C47" s="7"/>
       <c r="D47" s="5"/>
       <c r="E47" s="6"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="8"/>
       <c r="B48" s="8"/>
       <c r="C48" s="7"/>

</xml_diff>